<commit_message>
docs: rebuild all three files with em dashes removed
- genomebridge_company_brief.pdf - all em/en dashes replaced with hyphens or plain text
- project_helix_key_requirements.pdf - all em/en dashes removed
- product_risk_register.xlsx - all em/en dashes removed, formulas clean (48 formulas, 0 errors)

HELIX-002
</commit_message>
<xml_diff>
--- a/docs/quality-strategy/product_risk_register.xlsx
+++ b/docs/quality-strategy/product_risk_register.xlsx
@@ -28,10 +28,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="272">
   <si>
-    <t xml:space="preserve">PROJECT HELIX — PRODUCT QUALITY RISK REGISTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GenomeBridge Clinical Systems Ltd  |  Phase 1 — Quality Discovery  |  Version 1.0  |  4 August 2026</t>
+    <t xml:space="preserve">PROJECT HELIX - PRODUCT QUALITY RISK REGISTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GenomeBridge Clinical Systems Ltd  |  Phase 1 - Quality Discovery  |  Version 1.0  |  4 August 2026</t>
   </si>
   <si>
     <t xml:space="preserve">Risk ID</t>
@@ -50,15 +50,15 @@
   </si>
   <si>
     <t xml:space="preserve">Likelihood
-(1–5)</t>
+(1-5)</t>
   </si>
   <si>
     <t xml:space="preserve">Impact
-(1–5)</t>
+(1-5)</t>
   </si>
   <si>
     <t xml:space="preserve">Risk Score
-(L×I)</t>
+(L x I)</t>
   </si>
   <si>
     <t xml:space="preserve">RAG</t>
@@ -96,7 +96,7 @@
     <t xml:space="preserve">Users search for a patient and select the wrong record because names or DOBs are similar</t>
   </si>
   <si>
-    <t xml:space="preserve">Step 1 — Locate patient</t>
+    <t xml:space="preserve">Step 1 - Locate patient</t>
   </si>
   <si>
     <t xml:space="preserve">Incorrect patient receives clinical referral or genomic test order</t>
@@ -120,10 +120,10 @@
     <t xml:space="preserve">Observed in OpenMRS: search returns multiple results with similar surnames</t>
   </si>
   <si>
-    <t xml:space="preserve">DCB0129 §6.3 — Hazard: wrong patient selected</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Priority 1 — feeds Phase 2 Charter 2</t>
+    <t xml:space="preserve">DCB0129 s6.3 - Hazard: wrong patient selected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Priority 1 - feeds Phase 2 Charter 2</t>
   </si>
   <si>
     <t xml:space="preserve">QR-002</t>
@@ -132,10 +132,10 @@
     <t xml:space="preserve">Duplicate Records</t>
   </si>
   <si>
-    <t xml:space="preserve">Two records are created for the same patient — one from registration, one from referral import</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Step 1 — Register patient</t>
+    <t xml:space="preserve">Two records are created for the same patient - one from registration, one from referral import</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step 1 - Register patient</t>
   </si>
   <si>
     <t xml:space="preserve">Duplicate referrals, split history, incorrect cumulative reporting</t>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">HAPI FHIR: conditional-create tested in Phase 3</t>
   </si>
   <si>
-    <t xml:space="preserve">DCB0129 §6.3 — Hazard: duplicate patient identity</t>
+    <t xml:space="preserve">DCB0129 s6.3 - Hazard: duplicate patient identity</t>
   </si>
   <si>
     <t xml:space="preserve">Phase 3 task: POST Patient with If-None-Exist header</t>
@@ -165,10 +165,10 @@
     <t xml:space="preserve">Incomplete Demographics</t>
   </si>
   <si>
-    <t xml:space="preserve">Patient records are created with mandatory demographic fields missing — name, DOB or gender absent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Step 2 — Review demographics</t>
+    <t xml:space="preserve">Patient records are created with mandatory demographic fields missing - name, DOB or gender absent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step 2 - Review demographics</t>
   </si>
   <si>
     <t xml:space="preserve">Downstream referral validation fails; reports exclude patients</t>
@@ -192,7 +192,7 @@
     <t xml:space="preserve">None direct</t>
   </si>
   <si>
-    <t xml:space="preserve">Boundary-value analysis on DOB field — Phase 2 task</t>
+    <t xml:space="preserve">Boundary-value analysis on DOB field - Phase 2 task</t>
   </si>
   <si>
     <t xml:space="preserve">QR-004</t>
@@ -204,7 +204,7 @@
     <t xml:space="preserve">Genomic test request is created without a recorded consent resource</t>
   </si>
   <si>
-    <t xml:space="preserve">Step 4 — Record consent</t>
+    <t xml:space="preserve">Step 4 - Record consent</t>
   </si>
   <si>
     <t xml:space="preserve">Regulatory non-compliance; test request legally invalid</t>
@@ -219,7 +219,7 @@
     <t xml:space="preserve">FHIR Consent created and linked in Phase 3 workflow chain</t>
   </si>
   <si>
-    <t xml:space="preserve">DCB0129 §6.3 — Hazard: consent not obtained</t>
+    <t xml:space="preserve">DCB0129 s6.3 - Hazard: consent not obtained</t>
   </si>
   <si>
     <t xml:space="preserve">CONS-MISS code in operational queue report</t>
@@ -234,7 +234,7 @@
     <t xml:space="preserve">ServiceRequest records are submitted with one or more mandatory clinical fields absent</t>
   </si>
   <si>
-    <t xml:space="preserve">Step 3 — Create referral</t>
+    <t xml:space="preserve">Step 3 - Create referral</t>
   </si>
   <si>
     <t xml:space="preserve">Referral cannot be processed; TAT clock starts incorrectly</t>
@@ -261,7 +261,7 @@
     <t xml:space="preserve">Specimen resource is created but not correctly associated with its parent ServiceRequest</t>
   </si>
   <si>
-    <t xml:space="preserve">Step 6 — Associate specimen</t>
+    <t xml:space="preserve">Step 6 - Associate specimen</t>
   </si>
   <si>
     <t xml:space="preserve">Genomic test cannot proceed; specimen appears orphaned in queue</t>
@@ -279,10 +279,10 @@
     <t xml:space="preserve">SPEC-UNLINK is the primary metric thread across all phases</t>
   </si>
   <si>
-    <t xml:space="preserve">DCB0129 §6.3 — Hazard: wrong specimen used</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRIMARY RISK — answer key metric lives here</t>
+    <t xml:space="preserve">DCB0129 s6.3 - Hazard: wrong specimen used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRIMARY RISK - answer key metric lives here</t>
   </si>
   <si>
     <t xml:space="preserve">QR-007</t>
@@ -291,10 +291,10 @@
     <t xml:space="preserve">Workflow Status Tracking</t>
   </si>
   <si>
-    <t xml:space="preserve">Task resource status is not updated when processing moves between stages — WF-STALL accumulates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Step 7 — Track status</t>
+    <t xml:space="preserve">Task resource status is not updated when processing moves between stages - WF-STALL accumulates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step 7 - Track status</t>
   </si>
   <si>
     <t xml:space="preserve">Operational team cannot identify blocked referrals; SLA breached silently</t>
@@ -321,7 +321,7 @@
     <t xml:space="preserve">DiagnosticReport resource is created but not linked to the correct patient or subject</t>
   </si>
   <si>
-    <t xml:space="preserve">Step 8 — Diagnostic report</t>
+    <t xml:space="preserve">Step 8 - Diagnostic report</t>
   </si>
   <si>
     <t xml:space="preserve">Clinician retrieves wrong report or report is inaccessible</t>
@@ -336,10 +336,10 @@
     <t xml:space="preserve">DiagnosticReport relationship tested in Phase 3 chain</t>
   </si>
   <si>
-    <t xml:space="preserve">DCB0129 §6.3 — Hazard: wrong result attributed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low likelihood — tested for completeness of hazard coverage</t>
+    <t xml:space="preserve">DCB0129 s6.3 - Hazard: wrong result attributed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low likelihood - tested for completeness of hazard coverage</t>
   </si>
   <si>
     <t xml:space="preserve">QR-009</t>
@@ -351,7 +351,7 @@
     <t xml:space="preserve">A user in one role can access a patient record or referral they should not see</t>
   </si>
   <si>
-    <t xml:space="preserve">Step 9 — Access control</t>
+    <t xml:space="preserve">Step 9 - Access control</t>
   </si>
   <si>
     <t xml:space="preserve">Patient confidentiality breach; UK GDPR Article 5(1)(f) violation</t>
@@ -366,10 +366,10 @@
     <t xml:space="preserve">OpenMRS role exploration in Phase 2</t>
   </si>
   <si>
-    <t xml:space="preserve">DCB0160 §8 — Deploying organisation access controls</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Awareness only — cannot perform security testing against public system</t>
+    <t xml:space="preserve">DCB0160 s8 - Deploying organisation access controls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Awareness only - cannot perform security testing against public system</t>
   </si>
   <si>
     <t xml:space="preserve">QR-010</t>
@@ -381,7 +381,7 @@
     <t xml:space="preserve">An authenticated session does not terminate correctly on logout or timeout</t>
   </si>
   <si>
-    <t xml:space="preserve">Step 9 — Session</t>
+    <t xml:space="preserve">Step 9 - Session</t>
   </si>
   <si>
     <t xml:space="preserve">Subsequent user on shared terminal accesses prior session</t>
@@ -408,22 +408,22 @@
     <t xml:space="preserve">Validation messages are absent, inconsistent or misleading across registration and referral forms</t>
   </si>
   <si>
-    <t xml:space="preserve">Steps 1–3</t>
+    <t xml:space="preserve">Steps 1-3</t>
   </si>
   <si>
     <t xml:space="preserve">Users submit incomplete data believing it was accepted; support ticket volume increases</t>
   </si>
   <si>
-    <t xml:space="preserve">Cypress validation suite Phase 5 — equivalence partitioning and boundary-value analysis applied</t>
+    <t xml:space="preserve">Cypress validation suite Phase 5 - equivalence partitioning and boundary-value analysis applied</t>
   </si>
   <si>
     <t xml:space="preserve">Cypress Phase 5</t>
   </si>
   <si>
-    <t xml:space="preserve">Phase 2 charter 3 and 5 — validation behaviour documented</t>
-  </si>
-  <si>
-    <t xml:space="preserve">James Wright complaint theme — form validation issues</t>
+    <t xml:space="preserve">Phase 2 charter 3 and 5 - validation behaviour documented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">James Wright complaint theme - form validation issues</t>
   </si>
   <si>
     <t xml:space="preserve">QR-012</t>
@@ -435,7 +435,7 @@
     <t xml:space="preserve">A change to the FHIR API contract removes or renames a field, breaking downstream consumers</t>
   </si>
   <si>
-    <t xml:space="preserve">Steps 3–8 — all API consumers</t>
+    <t xml:space="preserve">Steps 3-8 - all API consumers</t>
   </si>
   <si>
     <t xml:space="preserve">Consumers silently receive null where a value is expected; data loss</t>
@@ -444,13 +444,13 @@
     <t xml:space="preserve">LOW</t>
   </si>
   <si>
-    <t xml:space="preserve">API compatibility analysis in Phase 3 — fictional old vs new contract diff</t>
+    <t xml:space="preserve">API compatibility analysis in Phase 3 - fictional old vs new contract diff</t>
   </si>
   <si>
     <t xml:space="preserve">Compatibility assessment document produced in Phase 3</t>
   </si>
   <si>
-    <t xml:space="preserve">Backwards-compatibility risk analysis — no live Pact environment required</t>
+    <t xml:space="preserve">Backwards-compatibility risk analysis - no live Pact environment required</t>
   </si>
   <si>
     <t xml:space="preserve">QR-013</t>
@@ -462,7 +462,7 @@
     <t xml:space="preserve">A synthetic record is created with a format indistinguishable from real patient data</t>
   </si>
   <si>
-    <t xml:space="preserve">All phases — test data</t>
+    <t xml:space="preserve">All phases - test data</t>
   </si>
   <si>
     <t xml:space="preserve">GDPR breach risk; regulatory non-compliance under UK DSPT</t>
@@ -471,10 +471,10 @@
     <t xml:space="preserve">Synthetic data policy produced in Phase 4; naming convention and tagging enforced</t>
   </si>
   <si>
-    <t xml:space="preserve">SQL Phase 4 — data policy + naming convention</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Laura Okafor constraint — non-negotiable</t>
+    <t xml:space="preserve">SQL Phase 4 - data policy + naming convention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laura Okafor constraint - non-negotiable</t>
   </si>
   <si>
     <t xml:space="preserve">UK GDPR Article 5 + NHS DSPT</t>
@@ -492,7 +492,7 @@
     <t xml:space="preserve">Key clinical workflows are inaccessible to users relying on keyboard navigation or assistive technology</t>
   </si>
   <si>
-    <t xml:space="preserve">Steps 1–3 — patient search and registration</t>
+    <t xml:space="preserve">Steps 1-3 - patient search and registration</t>
   </si>
   <si>
     <t xml:space="preserve">Clinical staff with accessibility needs cannot complete referral workflow</t>
@@ -504,10 +504,10 @@
     <t xml:space="preserve">Exploratory Phase 2 + Playwright Phase 6 (axe-core)</t>
   </si>
   <si>
-    <t xml:space="preserve">Phase 2 charter 7 — keyboard-only workflow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WCAG 2.1 AA — not DCB0129 directly</t>
+    <t xml:space="preserve">Phase 2 charter 7 - keyboard-only workflow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WCAG 2.1 AA - not DCB0129 directly</t>
   </si>
   <si>
     <t xml:space="preserve">Niche but recurring in UK healthtech QA postings</t>
@@ -525,13 +525,13 @@
     <t xml:space="preserve">Clinical users on non-Chrome browsers experience broken workflows</t>
   </si>
   <si>
-    <t xml:space="preserve">Playwright cross-browser Phase 6 — Journey 3 runs in Chromium, Firefox and WebKit</t>
+    <t xml:space="preserve">Playwright cross-browser Phase 6 - Journey 3 runs in Chromium, Firefox and WebKit</t>
   </si>
   <si>
     <t xml:space="preserve">Playwright Phase 6</t>
   </si>
   <si>
-    <t xml:space="preserve">Phase 2 charter 8 — browser behaviour documented</t>
+    <t xml:space="preserve">Phase 2 charter 8 - browser behaviour documented</t>
   </si>
   <si>
     <t xml:space="preserve">Environmental failures must be distinguished from genuine defects</t>
@@ -552,10 +552,10 @@
     <t xml:space="preserve">False confidence in green build; real defects masked by flaky tests</t>
   </si>
   <si>
-    <t xml:space="preserve">Phase 5 reliability measurement — first-run vs final pass rate; flaky-test root-cause analysis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cypress Phase 5 — reliability analysis</t>
+    <t xml:space="preserve">Phase 5 reliability measurement - first-run vs final pass rate; flaky-test root-cause analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cypress Phase 5 - reliability analysis</t>
   </si>
   <si>
     <t xml:space="preserve">Mark Evans handover acknowledges inconsistent standards</t>
@@ -582,7 +582,7 @@
     <t xml:space="preserve">Tests create own data dynamically; avoid fixed IDs; tolerate resets; CI timeout controls; environment instability classified separately from product defects</t>
   </si>
   <si>
-    <t xml:space="preserve">All phases — responsible testing rules enforced</t>
+    <t xml:space="preserve">All phases - responsible testing rules enforced</t>
   </si>
   <si>
     <t xml:space="preserve">Documented in Phase 7 CI/CD failure classification</t>
@@ -597,10 +597,10 @@
     <t xml:space="preserve">Test Data Reuse</t>
   </si>
   <si>
-    <t xml:space="preserve">Automation tests share a fixed patient record — one test's state change breaks subsequent tests</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phases 5 and 6 — automation</t>
+    <t xml:space="preserve">Automation tests share a fixed patient record - one test state change breaks subsequent tests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phases 5 and 6 - automation</t>
   </si>
   <si>
     <t xml:space="preserve">Non-deterministic failures; order-dependent test results</t>
@@ -630,13 +630,13 @@
     <t xml:space="preserve">Referral submission times out; clinical users abandon and retry creating duplicates</t>
   </si>
   <si>
-    <t xml:space="preserve">k6 performance tests against local mock endpoint in Phase 7 — baseline, expected load, stress spike, recovery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phase 7 — k6 performance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Local mock only — must not load-test public systems</t>
+    <t xml:space="preserve">k6 performance tests against local mock endpoint in Phase 7 - baseline, expected load, stress spike, recovery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase 7 - k6 performance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Local mock only - must not load-test public systems</t>
   </si>
   <si>
     <t xml:space="preserve">p50/p95/p99 latency thresholds defined in Phase 7</t>
@@ -651,7 +651,7 @@
     <t xml:space="preserve">Release decision is made based on raw test-pass count rather than risk-weighted quality evidence</t>
   </si>
   <si>
-    <t xml:space="preserve">Step — Release review</t>
+    <t xml:space="preserve">Step - Release review</t>
   </si>
   <si>
     <t xml:space="preserve">P1 defects ship to production because scorecard looked green</t>
@@ -660,16 +660,16 @@
     <t xml:space="preserve">Phase 8 final quality scorecard reconciles all phase evidence; Go/No-Go recommendation requires evidence per risk</t>
   </si>
   <si>
-    <t xml:space="preserve">Phase 8 — release readiness</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Addresses GenomeBridge's stated problem: 'release decisions rely too heavily on test count'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DCB0129 §9 — release authorisation requires documented evidence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Senior-stretch deliverable — Phase 8</t>
+    <t xml:space="preserve">Phase 8 - release readiness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Addresses GenomeBridge stated problem: release decisions rely too heavily on test count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DCB0129 s9 - release authorisation requires documented evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Senior-stretch deliverable - Phase 8</t>
   </si>
   <si>
     <t xml:space="preserve">QR-021</t>
@@ -681,7 +681,7 @@
     <t xml:space="preserve">QA evidence is presented to clinical safety reviewers without distinguishing what it does and does not prove</t>
   </si>
   <si>
-    <t xml:space="preserve">All phases — reporting</t>
+    <t xml:space="preserve">All phases - reporting</t>
   </si>
   <si>
     <t xml:space="preserve">Clinical Safety Officer makes assurance decisions on insufficient evidence</t>
@@ -696,10 +696,10 @@
     <t xml:space="preserve">DCB0129/DCB0160 awareness documented in company brief</t>
   </si>
   <si>
-    <t xml:space="preserve">DCB0129 §6 and DCB0160 §8 — clinical safety case ownership</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Awareness-level only — candidate is NOT the Clinical Safety Officer</t>
+    <t xml:space="preserve">DCB0129 s6 and DCB0160 s8 - clinical safety case ownership</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Awareness-level only - candidate is NOT the Clinical Safety Officer</t>
   </si>
   <si>
     <t xml:space="preserve">QR-022</t>
@@ -708,7 +708,7 @@
     <t xml:space="preserve">Traceability</t>
   </si>
   <si>
-    <t xml:space="preserve">Test results cannot be traced back to requirements or risks — release decision is not auditable</t>
+    <t xml:space="preserve">Test results cannot be traced back to requirements or risks - release decision is not auditable</t>
   </si>
   <si>
     <t xml:space="preserve">All phases</t>
@@ -720,19 +720,19 @@
     <t xml:space="preserve">Requirements traceability matrix built in Phase 1; updated each phase; final matrix in Phase 8</t>
   </si>
   <si>
-    <t xml:space="preserve">All phases — traceability matrix</t>
+    <t xml:space="preserve">All phases - traceability matrix</t>
   </si>
   <si>
     <t xml:space="preserve">Traceability matrix column present in this register</t>
   </si>
   <si>
-    <t xml:space="preserve">DCB0129 §9 — traceability of safety-relevant testing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cross-phase artefact — connects risk IDs to test IDs to evidence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PROJECT HELIX — RISK SUMMARY DASHBOARD</t>
+    <t xml:space="preserve">DCB0129 s9 - traceability of safety-relevant testing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cross-phase artefact - connects risk IDs to test IDs to evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROJECT HELIX - RISK SUMMARY DASHBOARD</t>
   </si>
   <si>
     <t xml:space="preserve">RAG Status</t>
@@ -744,19 +744,19 @@
     <t xml:space="preserve">Count</t>
   </si>
   <si>
-    <t xml:space="preserve">HIGH (≥16)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MEDIUM (9–15)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LOW (&lt;9)</t>
+    <t xml:space="preserve">HIGH (16 and above)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MEDIUM (9 to 15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOW (below 9)</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL RISKS</t>
   </si>
   <si>
-    <t xml:space="preserve">PROJECT HELIX — TEST LAYER DECISION MATRIX</t>
+    <t xml:space="preserve">PROJECT HELIX - TEST LAYER DECISION MATRIX</t>
   </si>
   <si>
     <t xml:space="preserve">Risk Statement (short)</t>
@@ -787,7 +787,7 @@
     <t xml:space="preserve">Wrong patient selected</t>
   </si>
   <si>
-    <t xml:space="preserve">✓</t>
+    <t xml:space="preserve">Y</t>
   </si>
   <si>
     <t xml:space="preserve">Duplicate patient records</t>

</xml_diff>